<commit_message>
Version 1.1.0 with binaries.
</commit_message>
<xml_diff>
--- a/test/test1.xlsx
+++ b/test/test1.xlsx
@@ -7,7 +7,8 @@
     <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
+    <sheet name="Scenes" sheetId="1" r:id="rId4"/>
+    <sheet name="Statistics" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -15,68 +16,93 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="26">
+  <si>
+    <t>#</t>
+  </si>
   <si>
     <t>Scene</t>
   </si>
   <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Where</t>
+  </si>
+  <si>
+    <t>Goal</t>
+  </si>
+  <si>
+    <t>Like, Words, man.</t>
+  </si>
+  <si>
+    <t>Synopsis</t>
+  </si>
+  <si>
+    <t>Earth</t>
+  </si>
+  <si>
+    <t>Making a Scene</t>
+  </si>
+  <si>
+    <t>1st Draft</t>
+  </si>
+  <si>
+    <t>Demonstrate that it’s worth exploring the next scene</t>
+  </si>
+  <si>
+    <t>Another Scene</t>
+  </si>
+  <si>
+    <t>More Scenes</t>
+  </si>
+  <si>
+    <t>An embedded scene</t>
+  </si>
+  <si>
+    <t>Space</t>
+  </si>
+  <si>
+    <t>Jane Cannot Find John</t>
+  </si>
+  <si>
+    <t>We Found John!</t>
+  </si>
+  <si>
+    <t>2nd Draft</t>
+  </si>
+  <si>
+    <t>Mars</t>
+  </si>
+  <si>
+    <t>Scene One</t>
+  </si>
+  <si>
+    <t>3rd Draft</t>
+  </si>
+  <si>
+    <t>Scenes</t>
+  </si>
+  <si>
     <t>Words</t>
   </si>
   <si>
-    <t>Point of View</t>
-  </si>
-  <si>
-    <t>Location(s)</t>
-  </si>
-  <si>
-    <t>Focus Character</t>
-  </si>
-  <si>
-    <t>Characters</t>
-  </si>
-  <si>
-    <t>Mentions</t>
-  </si>
-  <si>
-    <t>Jane</t>
-  </si>
-  <si>
-    <t>Earth</t>
-  </si>
-  <si>
-    <t>Making a Scene</t>
-  </si>
-  <si>
-    <t>John
-Jane</t>
-  </si>
-  <si>
-    <t>Space</t>
-  </si>
-  <si>
-    <t>Another Scene</t>
-  </si>
-  <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>Jane Cannot Find John</t>
-  </si>
-  <si>
-    <t>We Found John!</t>
-  </si>
-  <si>
-    <t>Mars</t>
-  </si>
-  <si>
-    <t>Scene One</t>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Inactive</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0!"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <b val="0"/>
@@ -117,19 +143,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
+    <xf xfId="0" fontId="0" numFmtId="164" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="164" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    <xf xfId="0" fontId="1" numFmtId="164" fillId="0" borderId="0" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -430,15 +465,16 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="21" customWidth="true" style="0"/>
-    <col min="2" max="2" width="7" customWidth="true" style="0"/>
-    <col min="3" max="3" width="19" customWidth="true" style="0"/>
-    <col min="4" max="4" width="16" customWidth="true" style="0"/>
-    <col min="5" max="5" width="21" customWidth="true" style="0"/>
-    <col min="6" max="6" width="14" customWidth="true" style="0"/>
+    <col min="1" max="1" width="2" customWidth="true" style="0"/>
+    <col min="2" max="2" width="22" customWidth="true" style="0"/>
+    <col min="3" max="3" width="10" customWidth="true" style="0"/>
+    <col min="4" max="4" width="7" customWidth="true" style="0"/>
+    <col min="5" max="5" width="55" customWidth="true" style="0"/>
+    <col min="6" max="6" width="24" customWidth="true" style="0"/>
+    <col min="7" max="7" width="12" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -465,96 +501,295 @@
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="C2" s="2" t="s">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="C3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="4">
+        <v>534</v>
+      </c>
+      <c r="G3" s="2"/>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="4">
+        <v>79</v>
+      </c>
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="2">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="4">
+        <v>420</v>
+      </c>
+      <c r="G5" s="2"/>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="2">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="4">
+        <v>7</v>
+      </c>
+      <c r="G6" s="2"/>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="2">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="4">
+        <v>21</v>
+      </c>
+      <c r="G7" s="2"/>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="2">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="2"/>
+      <c r="F8" s="4">
+        <v>34</v>
+      </c>
+      <c r="G8" s="2"/>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="2">
+        <v>1</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="4">
+        <v>51</v>
+      </c>
+      <c r="G9" s="2"/>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="F10" s="6">
+        <v>1146</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="12.6" customWidth="true" style="0"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="B1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="4">
-        <v>530</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="B3" s="6">
+        <v>5</v>
+      </c>
+      <c r="C3" s="6">
+        <v>0</v>
+      </c>
+      <c r="D3" s="7">
+        <v>5</v>
+      </c>
+      <c r="E3" s="6">
+        <v>1061</v>
+      </c>
+      <c r="F3" s="6">
+        <v>0</v>
+      </c>
+      <c r="G3" s="7">
+        <v>1061</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="6">
+        <v>1</v>
+      </c>
+      <c r="C4" s="6">
+        <v>0</v>
+      </c>
+      <c r="D4" s="7">
+        <v>1</v>
+      </c>
+      <c r="E4" s="6">
+        <v>34</v>
+      </c>
+      <c r="F4" s="6">
+        <v>0</v>
+      </c>
+      <c r="G4" s="7">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="6">
+        <v>1</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0</v>
+      </c>
+      <c r="D5" s="7">
+        <v>1</v>
+      </c>
+      <c r="E5" s="6">
+        <v>51</v>
+      </c>
+      <c r="F5" s="6">
+        <v>0</v>
+      </c>
+      <c r="G5" s="7">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="6">
         <v>7</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="4">
-        <v>108</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="C6" s="6">
+        <v>0</v>
+      </c>
+      <c r="D6" s="7">
         <v>7</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="4">
-        <v>28</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="4">
-        <v>37</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="4">
-        <v>55</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>13</v>
+      <c r="E6" s="6">
+        <v>1146</v>
+      </c>
+      <c r="F6" s="6">
+        <v>0</v>
+      </c>
+      <c r="G6" s="7">
+        <v>1146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Account for "allow repeated named comments" coming in nW 2.8
</commit_message>
<xml_diff>
--- a/test/test1.xlsx
+++ b/test/test1.xlsx
@@ -16,53 +16,152 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="26">
-  <si>
-    <t>#</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="56">
+  <si>
+    <t>Active</t>
   </si>
   <si>
     <t>Scene</t>
   </si>
   <si>
+    <t>Words</t>
+  </si>
+  <si>
     <t>Status</t>
   </si>
   <si>
-    <t>Where</t>
+    <t>Synopsis</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>Inciting Incident</t>
   </si>
   <si>
     <t>Goal</t>
   </si>
   <si>
-    <t>Like, Words, man.</t>
-  </si>
-  <si>
-    <t>Synopsis</t>
+    <t>Complication(s)</t>
+  </si>
+  <si>
+    <t>Turning Point</t>
+  </si>
+  <si>
+    <t>Crisis</t>
+  </si>
+  <si>
+    <t>(Non-)Resolution</t>
+  </si>
+  <si>
+    <t>Point of View</t>
+  </si>
+  <si>
+    <t>Period/Time</t>
+  </si>
+  <si>
+    <t>Duration</t>
+  </si>
+  <si>
+    <t>Location(s)</t>
+  </si>
+  <si>
+    <t>Focus Character</t>
+  </si>
+  <si>
+    <t>Characters</t>
+  </si>
+  <si>
+    <t>Mentions</t>
+  </si>
+  <si>
+    <t>Pace</t>
+  </si>
+  <si>
+    <t>What does it look like?</t>
+  </si>
+  <si>
+    <t>Quality/cadence in the prose</t>
+  </si>
+  <si>
+    <t>What are the characters feeling emotionally?</t>
+  </si>
+  <si>
+    <t>Jane</t>
   </si>
   <si>
     <t>Earth</t>
   </si>
   <si>
+    <t>yes</t>
+  </si>
+  <si>
     <t>Making a Scene</t>
   </si>
   <si>
     <t>1st Draft</t>
   </si>
   <si>
+    <t>Introduce new users to the basics of novelWriter</t>
+  </si>
+  <si>
+    <t>Someone installed novelWriter and opened the sample project</t>
+  </si>
+  <si>
     <t>Demonstrate that it’s worth exploring the next scene</t>
   </si>
   <si>
+    <t>Has previously used other software and is disoriented by the interface
+A new update allows duplicate tags of the same name</t>
+  </si>
+  <si>
+    <t>Realizes that Markdown syntax is actually very easy to understand and use.</t>
+  </si>
+  <si>
+    <t>Fears the reader needs to learn a completely new language, “Markdown”</t>
+  </si>
+  <si>
+    <t>Axniety about learning a new thing has been addressed.</t>
+  </si>
+  <si>
+    <t>5m</t>
+  </si>
+  <si>
+    <t>John
+Jane</t>
+  </si>
+  <si>
+    <t>Space</t>
+  </si>
+  <si>
+    <t>slow, informative</t>
+  </si>
+  <si>
+    <t>A nominally clean, sparse apartment in a high rise tower.</t>
+  </si>
+  <si>
+    <t>friendly although technical</t>
+  </si>
+  <si>
+    <t>bewilderment, fear.</t>
+  </si>
+  <si>
     <t>Another Scene</t>
   </si>
   <si>
+    <t>This is the first bit
+This is the second bit</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
     <t>More Scenes</t>
   </si>
   <si>
     <t>An embedded scene</t>
   </si>
   <si>
-    <t>Space</t>
-  </si>
-  <si>
     <t>Jane Cannot Find John</t>
   </si>
   <si>
@@ -82,12 +181,6 @@
   </si>
   <si>
     <t>Scenes</t>
-  </si>
-  <si>
-    <t>Words</t>
-  </si>
-  <si>
-    <t>Active</t>
   </si>
   <si>
     <t>Inactive</t>
@@ -100,9 +193,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0!"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <b val="0"/>
@@ -149,22 +240,22 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="164" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
+    <xf xfId="0" fontId="0" numFmtId="3" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="164" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="1" numFmtId="164" fillId="0" borderId="0" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    <xf xfId="0" fontId="1" numFmtId="3" fillId="0" borderId="0" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -465,19 +556,34 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:W10"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="2" customWidth="true" style="0"/>
-    <col min="2" max="2" width="22" customWidth="true" style="0"/>
-    <col min="3" max="3" width="10" customWidth="true" style="0"/>
-    <col min="4" max="4" width="7" customWidth="true" style="0"/>
-    <col min="5" max="5" width="55" customWidth="true" style="0"/>
-    <col min="6" max="6" width="24" customWidth="true" style="0"/>
-    <col min="7" max="7" width="12" customWidth="true" style="0"/>
+    <col min="1" max="1" width="9" customWidth="true" style="0"/>
+    <col min="2" max="2" width="21" customWidth="true" style="0"/>
+    <col min="3" max="3" width="7" customWidth="true" style="0"/>
+    <col min="4" max="4" width="9" customWidth="true" style="0"/>
+    <col min="5" max="5" width="22" customWidth="true" style="0"/>
+    <col min="6" max="6" width="40" customWidth="true" style="0"/>
+    <col min="7" max="7" width="40" customWidth="true" style="0"/>
+    <col min="8" max="8" width="40" customWidth="true" style="0"/>
+    <col min="9" max="9" width="40" customWidth="true" style="0"/>
+    <col min="10" max="10" width="40" customWidth="true" style="0"/>
+    <col min="11" max="11" width="40" customWidth="true" style="0"/>
+    <col min="12" max="12" width="40" customWidth="true" style="0"/>
+    <col min="13" max="13" width="19" customWidth="true" style="0"/>
+    <col min="14" max="14" width="16" customWidth="true" style="0"/>
+    <col min="15" max="15" width="12" customWidth="true" style="0"/>
+    <col min="16" max="16" width="16" customWidth="true" style="0"/>
+    <col min="17" max="17" width="21" customWidth="true" style="0"/>
+    <col min="18" max="18" width="14" customWidth="true" style="0"/>
+    <col min="19" max="19" width="12" customWidth="true" style="0"/>
+    <col min="20" max="20" width="17" customWidth="true" style="0"/>
+    <col min="21" max="21" width="40" customWidth="true" style="0"/>
+    <col min="22" max="22" width="40" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:23">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -499,155 +605,265 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="3" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="2"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="2">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23">
+      <c r="M2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23">
+      <c r="A3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="4">
+        <v>534</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" s="5">
+        <v>0</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="T3" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="U3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="V3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="W3" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="4">
+        <v>79</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23">
+      <c r="A5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="4">
+        <v>420</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q5" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23">
+      <c r="A6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="4">
         <v>7</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="4">
-        <v>534</v>
-      </c>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="2">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="2"/>
-      <c r="F4" s="4">
-        <v>79</v>
-      </c>
-      <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="2">
-        <v>3</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="4">
-        <v>420</v>
-      </c>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="2">
-        <v>4</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="D6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="4">
-        <v>7</v>
-      </c>
-      <c r="G6" s="2"/>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="2">
-        <v>5</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="4">
+        <v>27</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23">
+      <c r="A7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="4">
         <v>21</v>
       </c>
-      <c r="G7" s="2"/>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="2">
-        <v>6</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>17</v>
+      <c r="D7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q7" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23">
+      <c r="A8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="4">
+        <v>34</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="4">
-        <v>34</v>
-      </c>
-      <c r="G8" s="2"/>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="2">
-        <v>1</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="4">
+        <v>49</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23">
+      <c r="A9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G9" s="2"/>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="F10" s="6">
+      <c r="C9" s="4">
+        <v>51</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23">
+      <c r="C10" s="4">
         <v>1146</v>
       </c>
     </row>
@@ -671,52 +887,52 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>22</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="6">
+      <c r="A3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="4">
         <v>5</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="4">
         <v>0</v>
       </c>
       <c r="D3" s="7">
         <v>5</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="4">
         <v>1061</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="4">
         <v>0</v>
       </c>
       <c r="G3" s="7">
@@ -724,22 +940,22 @@
       </c>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="6">
+      <c r="A4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="4">
         <v>1</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="4">
         <v>0</v>
       </c>
       <c r="D4" s="7">
         <v>1</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="4">
         <v>34</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="4">
         <v>0</v>
       </c>
       <c r="G4" s="7">
@@ -747,22 +963,22 @@
       </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="6">
+      <c r="A5" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="4">
         <v>1</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="4">
         <v>0</v>
       </c>
       <c r="D5" s="7">
         <v>1</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="4">
         <v>51</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="4">
         <v>0</v>
       </c>
       <c r="G5" s="7">
@@ -770,22 +986,22 @@
       </c>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="6">
+      <c r="A6" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="4">
         <v>7</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="4">
         <v>0</v>
       </c>
       <c r="D6" s="7">
         <v>7</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="4">
         <v>1146</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="4">
         <v>0</v>
       </c>
       <c r="G6" s="7">

</xml_diff>